<commit_message>
feat: integrate DRS metrics into T20 data processing and update caveman-compress skill utilities
</commit_message>
<xml_diff>
--- a/local_match_ingestion_summary.xlsx
+++ b/local_match_ingestion_summary.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="League Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded Matches" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="League Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Excluded Matches" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
chore: update dashboard timestamps and refresh analytics datasets
</commit_message>
<xml_diff>
--- a/local_match_ingestion_summary.xlsx
+++ b/local_match_ingestion_summary.xlsx
@@ -532,10 +532,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="C5" t="n">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-12</t>
         </is>
       </c>
     </row>
@@ -555,10 +555,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="C6" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -567,7 +567,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add squad roster explorer, update DPL 2026 data source, and enable multi-player selection for batting performance metrics
</commit_message>
<xml_diff>
--- a/local_match_ingestion_summary.xlsx
+++ b/local_match_ingestion_summary.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="League Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Excluded Matches" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="League Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded Matches" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,10 +463,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="C2" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -475,7 +475,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2025-08-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: standardize team names for Purani Dilli 6 and update dashboard timestamps
</commit_message>
<xml_diff>
--- a/local_match_ingestion_summary.xlsx
+++ b/local_match_ingestion_summary.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="League Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded Matches" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="League Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Excluded Matches" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,10 +463,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>77</v>
+        <v>111</v>
       </c>
       <c r="C2" t="n">
-        <v>77</v>
+        <v>111</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -475,7 +475,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-30</t>
         </is>
       </c>
     </row>

</xml_diff>